<commit_message>
Change in AuSteel cvxlab problem
Y collapsed to one single column
</commit_message>
<xml_diff>
--- a/mario/tools/cvxlab/AuSteel/mapping.xlsx
+++ b/mario/tools/cvxlab/AuSteel/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/tools/cvxlab/AuSteel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BD17B49-F02B-458E-A744-3E43D2595772}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{9C095DC2-CC44-BD40-B88D-9DE0D7147A4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80E8E05D-74AA-4BA5-953B-AAFFA66D7C69}"/>
   <bookViews>
-    <workbookView xWindow="-10130" yWindow="-21710" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sets" sheetId="1" r:id="rId1"/>
@@ -187,9 +187,6 @@
     <t>sat_acc_Name, region_to_Name, activity_to_Name</t>
   </si>
   <si>
-    <t>region_from_Name, region_to_Name, commodity_from_Name, cons_categ_Name</t>
-  </si>
-  <si>
     <t>fact_prod_Name, region_to_Name, activity_to_Name</t>
   </si>
   <si>
@@ -199,13 +196,16 @@
     <t>region_from_Name, commodity_from_Name</t>
   </si>
   <si>
+    <t>row level</t>
+  </si>
+  <si>
+    <t>col level</t>
+  </si>
+  <si>
+    <t>region_from_Name, commodity_from_Name, region_to_Name, cons_categ_Name</t>
+  </si>
+  <si>
     <t>region_to_Name, cons_categ_Name</t>
-  </si>
-  <si>
-    <t>row level</t>
-  </si>
-  <si>
-    <t>col level</t>
   </si>
 </sst>
 </file>
@@ -825,10 +825,10 @@
         <v>43</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -842,7 +842,7 @@
         <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s">
         <v>22</v>
@@ -862,7 +862,7 @@
         <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
         <v>21</v>
@@ -879,10 +879,10 @@
         <v>34</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
         <v>51</v>
-      </c>
-      <c r="D4" t="s">
-        <v>52</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
@@ -899,10 +899,10 @@
         <v>0</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
         <v>22</v>
@@ -922,7 +922,7 @@
         <v>49</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E6" t="s">
         <v>8</v>

</xml_diff>